<commit_message>
Update Gantt chart and add project folders
</commit_message>
<xml_diff>
--- a/Planning/BrickBuster-GanttChart.xlsx
+++ b/Planning/BrickBuster-GanttChart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arghi\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB7F7693-DE75-4D39-A34B-95F3300421BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{476A09F3-F1E6-4F11-BF27-921F60A851EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="67">
   <si>
     <t>Colours: Arghi = blue; Numan = green; Jack = purple; Ruth = amber; shared = grey; submission = red.</t>
   </si>
@@ -86,9 +86,6 @@
     <t>None</t>
   </si>
   <si>
-    <t>Not recorded</t>
-  </si>
-  <si>
     <t>2</t>
   </si>
   <si>
@@ -233,10 +230,10 @@
     <t>Done</t>
   </si>
   <si>
-    <t>In progress</t>
-  </si>
-  <si>
     <t>Brick Buster Gantt Chart</t>
+  </si>
+  <si>
+    <t>Not started</t>
   </si>
 </sst>
 </file>
@@ -1030,7 +1027,7 @@
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="48" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E3" s="46"/>
       <c r="F3" s="46"/>
@@ -1274,7 +1271,7 @@
         <v>16</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J7" s="20"/>
       <c r="K7" s="21">
@@ -1374,10 +1371,10 @@
     </row>
     <row r="8" spans="1:35" ht="38" customHeight="1">
       <c r="A8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>18</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>19</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>14</v>
@@ -1396,10 +1393,10 @@
         <v>2</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="21">
@@ -1496,16 +1493,16 @@
     </row>
     <row r="9" spans="1:35" ht="38" customHeight="1">
       <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="C9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>23</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>24</v>
       </c>
       <c r="E9" s="5">
         <v>46293</v>
@@ -1518,10 +1515,10 @@
         <v>4</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="J9" s="1"/>
       <c r="K9" s="21">
@@ -1615,10 +1612,10 @@
     </row>
     <row r="10" spans="1:35" ht="38" customHeight="1">
       <c r="A10" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>26</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>27</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>14</v>
@@ -1637,10 +1634,10 @@
         <v>4</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="J10" s="1"/>
       <c r="K10" s="21">
@@ -1734,13 +1731,13 @@
     </row>
     <row r="11" spans="1:35" ht="38" customHeight="1">
       <c r="A11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="C11" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>31</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>15</v>
@@ -1756,10 +1753,10 @@
         <v>4</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="J11" s="1"/>
       <c r="K11" s="21">
@@ -1853,16 +1850,16 @@
     </row>
     <row r="12" spans="1:35" ht="38" customHeight="1">
       <c r="A12" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="13" t="s">
-        <v>34</v>
-      </c>
       <c r="C12" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>23</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>24</v>
       </c>
       <c r="E12" s="5">
         <v>46297</v>
@@ -1875,10 +1872,10 @@
         <v>5</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="J12" s="1"/>
       <c r="K12" s="21">
@@ -1969,16 +1966,16 @@
     </row>
     <row r="13" spans="1:35" ht="38" customHeight="1">
       <c r="A13" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="C13" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>38</v>
-      </c>
       <c r="D13" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E13" s="5">
         <v>46297</v>
@@ -1991,10 +1988,10 @@
         <v>5</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="J13" s="1"/>
       <c r="K13" s="21">
@@ -2085,13 +2082,13 @@
     </row>
     <row r="14" spans="1:35" ht="38" customHeight="1">
       <c r="A14" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="14" t="s">
-        <v>41</v>
-      </c>
       <c r="C14" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>14</v>
@@ -2107,10 +2104,10 @@
         <v>5</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="J14" s="1"/>
       <c r="K14" s="21">
@@ -2198,10 +2195,10 @@
     </row>
     <row r="15" spans="1:35" ht="38" customHeight="1">
       <c r="A15" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="15" t="s">
         <v>42</v>
-      </c>
-      <c r="B15" s="15" t="s">
-        <v>43</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>15</v>
@@ -2220,10 +2217,10 @@
         <v>1</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="J15" s="1"/>
       <c r="K15" s="21">
@@ -2326,16 +2323,16 @@
     </row>
     <row r="16" spans="1:35" ht="38" customHeight="1">
       <c r="A16" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="C16" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="9" t="s">
         <v>46</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>47</v>
       </c>
       <c r="E16" s="5">
         <v>46302</v>
@@ -2348,10 +2345,10 @@
         <v>5</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="J16" s="1"/>
       <c r="K16" s="21">
@@ -2442,16 +2439,16 @@
     </row>
     <row r="17" spans="1:35" ht="38" customHeight="1">
       <c r="A17" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="B17" s="12" t="s">
-        <v>50</v>
-      </c>
       <c r="C17" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E17" s="5">
         <v>46302</v>
@@ -2464,10 +2461,10 @@
         <v>5</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="J17" s="1"/>
       <c r="K17" s="21">
@@ -2558,13 +2555,13 @@
     </row>
     <row r="18" spans="1:35" ht="38" customHeight="1">
       <c r="A18" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="C18" s="9" t="s">
         <v>52</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>53</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>15</v>
@@ -2580,10 +2577,10 @@
         <v>3</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="J18" s="1"/>
       <c r="K18" s="21">
@@ -2680,10 +2677,10 @@
     </row>
     <row r="19" spans="1:35" ht="38" customHeight="1">
       <c r="A19" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="15" t="s">
         <v>55</v>
-      </c>
-      <c r="B19" s="15" t="s">
-        <v>56</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>15</v>
@@ -2702,10 +2699,10 @@
         <v>2</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="J19" s="1"/>
       <c r="K19" s="21">
@@ -2805,10 +2802,10 @@
     </row>
     <row r="20" spans="1:35" ht="38" customHeight="1">
       <c r="A20" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>58</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>59</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>14</v>
@@ -2827,10 +2824,10 @@
         <v>1</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="J20" s="1"/>
       <c r="K20" s="21">
@@ -2933,16 +2930,16 @@
     </row>
     <row r="21" spans="1:35" ht="38" customHeight="1">
       <c r="A21" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21" s="18" t="s">
         <v>61</v>
-      </c>
-      <c r="B21" s="18" t="s">
-        <v>62</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E21" s="5">
         <v>46311</v>
@@ -2955,10 +2952,10 @@
         <v>1</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="J21" s="1"/>
       <c r="K21" s="21">

</xml_diff>